<commit_message>
docs: add TC05 problem_user image validation
</commit_message>
<xml_diff>
--- a/test case/Saucedemo test using playwright.xlsx
+++ b/test case/Saucedemo test using playwright.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -455,6 +455,47 @@
       <t xml:space="preserve"> 
 7. User is able to see backpack in "Your cart" list</t>
     </r>
+  </si>
+  <si>
+    <t>TC05</t>
+  </si>
+  <si>
+    <t>The objective of this test case is to validate the login function and UI rendering for the problem_user account.</t>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">1. Open </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>https://www.saucedemo.com/</t>
+    </r>
+    <r>
+      <rPr/>
+      <t xml:space="preserve"> 
+2. Input "problem_user" username
+3. Input correct password
+4. Select login
+5. Validate product images load correctly</t>
+    </r>
+  </si>
+  <si>
+    <t>1. https://www.saucedemo.com/ opens successfully
+2. Username input
+3. Password input
+4. Login button clicked and inventory page is visible
+5. All product images display correct artwork</t>
+  </si>
+  <si>
+    <t>1. https://www.saucedemo.com/ opens successfully
+2. Username input
+3. Password input
+4. Login button clicked and inventory page is visible
+5. AProduct images show incorrect image (dog picture) for all products.</t>
   </si>
 </sst>
 </file>
@@ -478,34 +519,57 @@
       <color rgb="FF0000FF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -753,79 +817,96 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -845,7 +926,8 @@
     <hyperlink r:id="rId14" ref="C5"/>
     <hyperlink r:id="rId15" ref="D5"/>
     <hyperlink r:id="rId16" ref="E5"/>
+    <hyperlink r:id="rId17" ref="C6"/>
   </hyperlinks>
-  <drawing r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>